<commit_message>
feat: enrich company funding profiles
</commit_message>
<xml_diff>
--- a/近期融资公司追踪.xlsx
+++ b/近期融资公司追踪.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R7dac3b90c819402e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="R9b07c60d7aba4f5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="Rfeefbbf48dea4ce6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R485f2d88792e46fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rfb38952673ad4064"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R0379aa3fd5e648ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -331,6 +331,9 @@
     <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -347,6 +350,9 @@
       <x:c r="I1" s="4"/>
       <x:c r="J1" s="4"/>
       <x:c r="K1" s="4"/>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="4"/>
+      <x:c r="N1" s="4"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -362,6 +368,9 @@
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7"/>
       <x:c r="K2" s="7"/>
+      <x:c r="L2" s="7"/>
+      <x:c r="M2" s="7"/>
+      <x:c r="N2" s="7"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -397,6 +406,15 @@
       <x:c r="K4" s="11" t="str">
         <x:v>核验状态</x:v>
       </x:c>
+      <x:c r="L4" s="11" t="str">
+        <x:v>企业介绍</x:v>
+      </x:c>
+      <x:c r="M4" s="11" t="str">
+        <x:v>企业网址</x:v>
+      </x:c>
+      <x:c r="N4" s="11" t="str">
+        <x:v>公开联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -432,6 +450,15 @@
       <x:c r="K5" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L5" s="12" t="str">
+        <x:v>企业级 AI 基础设施公司，围绕数据管理与 AI 计算场景提供技术产品。</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
+        <x:v>https://www.matrixorigin.cn/</x:v>
+      </x:c>
+      <x:c r="N5" s="12" t="str">
+        <x:v>商务联系：官网联系页</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -465,6 +492,15 @@
       <x:c r="K6" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L6" s="12" t="str">
+        <x:v>为光能源 是一家专注于电力电子 / 固态变压器的企业。</x:v>
+      </x:c>
+      <x:c r="M6" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N6" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -498,6 +534,15 @@
       <x:c r="K7" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L7" s="12" t="str">
+        <x:v>飞捷科思 是一家专注于半导体的企业。</x:v>
+      </x:c>
+      <x:c r="M7" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N7" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
@@ -531,6 +576,15 @@
       <x:c r="K8" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L8" s="12" t="str">
+        <x:v>蓝凌星通 是一家专注于卫星通信的企业。</x:v>
+      </x:c>
+      <x:c r="M8" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N8" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
@@ -564,6 +618,15 @@
       <x:c r="K9" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L9" s="12" t="str">
+        <x:v>昉擎科技 是一家专注于AI 算力芯片的企业。</x:v>
+      </x:c>
+      <x:c r="M9" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N9" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
@@ -597,6 +660,15 @@
       <x:c r="K10" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L10" s="12" t="str">
+        <x:v>协鑫光电 是一家专注于钙钛矿光伏的企业。</x:v>
+      </x:c>
+      <x:c r="M10" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N10" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
@@ -632,6 +704,15 @@
       <x:c r="K11" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L11" s="12" t="str">
+        <x:v>主动科技 是一家专注于脑机接口的企业。</x:v>
+      </x:c>
+      <x:c r="M11" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N11" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -665,6 +746,15 @@
       <x:c r="K12" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L12" s="12" t="str">
+        <x:v>生成式 AI 公司，聚焦多模态大模型与 AI 原生应用研发。</x:v>
+      </x:c>
+      <x:c r="M12" s="12" t="str">
+        <x:v>https://www.westlake.ai/</x:v>
+      </x:c>
+      <x:c r="N12" s="12" t="str">
+        <x:v>商务联系：官网联系页</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
@@ -698,6 +788,15 @@
       <x:c r="K13" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L13" s="12" t="str">
+        <x:v>璨辰科技 是一家专注于医疗 AI / 虚拟器官仿真的企业。</x:v>
+      </x:c>
+      <x:c r="M13" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N13" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -733,6 +832,15 @@
       <x:c r="K14" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L14" s="12" t="str">
+        <x:v>鸿鹄航空 是一家专注于航空航天的企业。</x:v>
+      </x:c>
+      <x:c r="M14" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N14" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
@@ -768,46 +876,274 @@
       <x:c r="K15" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L15" s="12" t="str">
+        <x:v>元育生物 是一家专注于生物医药的企业。</x:v>
+      </x:c>
+      <x:c r="M15" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N15" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
+        <x:v>幺正量子</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>量子计算</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>数亿元人民币</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="str">
+        <x:v>A 轮</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="12" t="str">
+        <x:v>大河财立方</x:v>
+      </x:c>
+      <x:c r="I16" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J16" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K16" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L16" s="12" t="str">
+        <x:v>量子计算技术公司，面向量子软硬件与产业化应用开展研发。</x:v>
+      </x:c>
+      <x:c r="M16" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N16" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="12" t="str">
+        <x:v>恺望数据</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>AI 数据服务</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="str">
+        <x:v>逾亿元人民币</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="F17" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="12" t="str">
+        <x:v>封面新闻</x:v>
+      </x:c>
+      <x:c r="I17" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J17" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K17" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L17" s="12" t="str">
+        <x:v>AI 数据服务公司，为具身智能等场景提供数据采集、处理与训练支持。</x:v>
+      </x:c>
+      <x:c r="M17" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N17" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>求是光谱</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>光谱检测</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="str">
+        <x:v>B++ 轮</x:v>
+      </x:c>
+      <x:c r="F18" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I18" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J18" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K18" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L18" s="12" t="str">
+        <x:v>光谱检测技术公司，面向工业与科研场景提供光谱相关产品和解决方案。</x:v>
+      </x:c>
+      <x:c r="M18" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N18" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>熵简科技</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>企业软件 / 数据智能</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="str">
+        <x:v>C 轮</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G19" s="14"/>
+      <x:c r="H19" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I19" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J19" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K19" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L19" s="12" t="str">
+        <x:v>企业级技术服务公司，聚焦数据智能与软件产品研发。</x:v>
+      </x:c>
+      <x:c r="M19" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N19" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="12" t="str">
+        <x:v>灏存科技</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>硬科技</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="n">
+        <x:v>46235.333333333336</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="str">
+        <x:v>A+ 轮</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G20" s="14"/>
+      <x:c r="H20" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I20" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J20" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K20" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L20" s="12" t="str">
+        <x:v>硬科技企业，公开报道披露其近期完成 A+ 轮融资。</x:v>
+      </x:c>
+      <x:c r="M20" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N20" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="12" t="str">
         <x:v>月之暗面（Kimi）</x:v>
       </x:c>
-      <x:c r="B16" s="12" t="str">
+      <x:c r="B21" s="12" t="str">
         <x:v>大模型</x:v>
       </x:c>
-      <x:c r="C16" s="13" t="n">
+      <x:c r="C21" s="13" t="n">
         <x:v>46234.333333333336</x:v>
       </x:c>
-      <x:c r="D16" s="12" t="str">
+      <x:c r="D21" s="12" t="str">
         <x:v>超 35 亿美元</x:v>
       </x:c>
-      <x:c r="E16" s="12" t="str">
+      <x:c r="E21" s="12" t="str">
         <x:v>F 轮</x:v>
       </x:c>
-      <x:c r="F16" s="12" t="str">
+      <x:c r="F21" s="12" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="G16" s="14" t="n">
+      <x:c r="G21" s="14" t="n">
         <x:v>2520000</x:v>
       </x:c>
-      <x:c r="H16" s="12" t="str">
+      <x:c r="H21" s="12" t="str">
         <x:v>创业邦</x:v>
       </x:c>
-      <x:c r="I16" s="16" t="str">
+      <x:c r="I21" s="16" t="str">
         <x:v>https://news.google.com/search?q=%E6%9C%88%E4%B9%8B%E6%9A%97%E9%9D%A2%20F%E8%BD%AE%2035%E4%BA%BF%E7%BE%8E%E5%85%83&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
-      <x:c r="J16" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
-      </x:c>
-      <x:c r="K16" s="12" t="str">
-        <x:v>已核验</x:v>
+      <x:c r="J21" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K21" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L21" s="12" t="str">
+        <x:v>大模型创业公司，推出 Kimi 等面向个人与企业的 AI 产品。</x:v>
+      </x:c>
+      <x:c r="M21" s="12" t="str">
+        <x:v>https://www.moonshot.cn/</x:v>
+      </x:c>
+      <x:c r="N21" s="12" t="str">
+        <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -828,6 +1164,9 @@
     <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -844,6 +1183,9 @@
       <x:c r="I1" s="4"/>
       <x:c r="J1" s="4"/>
       <x:c r="K1" s="4"/>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="4"/>
+      <x:c r="N1" s="4"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -859,6 +1201,9 @@
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7"/>
       <x:c r="K2" s="7"/>
+      <x:c r="L2" s="7"/>
+      <x:c r="M2" s="7"/>
+      <x:c r="N2" s="7"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -894,6 +1239,15 @@
       <x:c r="K4" s="11" t="str">
         <x:v>核验状态</x:v>
       </x:c>
+      <x:c r="L4" s="11" t="str">
+        <x:v>企业介绍</x:v>
+      </x:c>
+      <x:c r="M4" s="11" t="str">
+        <x:v>企业网址</x:v>
+      </x:c>
+      <x:c r="N4" s="11" t="str">
+        <x:v>公开联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -929,6 +1283,15 @@
       <x:c r="K5" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L5" s="12" t="str">
+        <x:v>Lumilens 是一家专注于光网络的企业。</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N5" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -964,6 +1327,15 @@
       <x:c r="K6" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L6" s="12" t="str">
+        <x:v>Valar Atomics 是一家专注于核能的企业。</x:v>
+      </x:c>
+      <x:c r="M6" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N6" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -999,6 +1371,15 @@
       <x:c r="K7" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L7" s="12" t="str">
+        <x:v>OLIX 是一家专注于AI 芯片的企业。</x:v>
+      </x:c>
+      <x:c r="M7" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N7" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
@@ -1034,6 +1415,15 @@
       <x:c r="K8" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L8" s="12" t="str">
+        <x:v>网络安全公司，提供以攻击路径验证为核心的安全测试与风险评估产品。</x:v>
+      </x:c>
+      <x:c r="M8" s="12" t="str">
+        <x:v>https://www.horizon3.ai/</x:v>
+      </x:c>
+      <x:c r="N8" s="12" t="str">
+        <x:v>商务联系：官网联系页</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
@@ -1069,11 +1459,20 @@
       <x:c r="K9" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
+      <x:c r="L9" s="12" t="str">
+        <x:v>AI Agent 安全公司，帮助企业识别和管控生成式 AI 与智能体的安全风险。</x:v>
+      </x:c>
+      <x:c r="M9" s="12" t="str">
+        <x:v>https://www.zenity.io/</x:v>
+      </x:c>
+      <x:c r="N9" s="12" t="str">
+        <x:v>商务联系：官网联系页</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1105,10 +1504,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46241.302557939816</x:v>
+        <x:v>46242.14893152778</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>12</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C2" t="n">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
data: add August seventh funding update
</commit_message>
<xml_diff>
--- a/近期融资公司追踪.xlsx
+++ b/近期融资公司追踪.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R485f2d88792e46fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rfb38952673ad4064"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R0379aa3fd5e648ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R7d386a9e909f4105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="R9724e5b4228a4776"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R95bc27f6f54e4fbe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -418,43 +418,41 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>矩阵起源</x:v>
+        <x:v>可灵 AI</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>企业级 AI 基础设施</x:v>
+        <x:v>AI 视频大模型</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46241.333333333336</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>超 1,000 万美元</x:v>
+        <x:v>近 30 亿美元</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="G5" s="14" t="n">
-        <x:v>7200</x:v>
-      </x:c>
+      <x:c r="G5" s="14"/>
       <x:c r="H5" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>新华网 / 经济参考报</x:v>
       </x:c>
       <x:c r="I5" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%9F%A9%E9%98%B5%E8%B5%B7%E6%BA%90%20%E8%B6%85%E5%8D%83%E4%B8%87%E7%BE%8E%E5%85%83%20A%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.news.cn/tech/20260807/1605ef446e5045b7ba0ee55245ce731c/c.html</x:v>
       </x:c>
       <x:c r="J5" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46242.48541666667</x:v>
       </x:c>
       <x:c r="K5" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L5" s="12" t="str">
-        <x:v>企业级 AI 基础设施公司，围绕数据管理与 AI 计算场景提供技术产品。</x:v>
+        <x:v>AI 视频大模型产品，面向内容创作和商业化视频生成场景提供服务。</x:v>
       </x:c>
       <x:c r="M5" s="12" t="str">
-        <x:v>https://www.matrixorigin.cn/</x:v>
+        <x:v>https://klingai.com/</x:v>
       </x:c>
       <x:c r="N5" s="12" t="str">
         <x:v>商务联系：官网联系页</x:v>
@@ -462,29 +460,31 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>为光能源</x:v>
+        <x:v>矩阵起源</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>电力电子 / 固态变压器</x:v>
+        <x:v>企业级 AI 基础设施</x:v>
       </x:c>
       <x:c r="C6" s="13" t="n">
         <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>超 1,000 万美元</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>B 轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G6" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="n">
+        <x:v>7200</x:v>
+      </x:c>
       <x:c r="H6" s="12" t="str">
-        <x:v>中国网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I6" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%BA%E5%85%89%E8%83%BD%E6%BA%90%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%9F%A9%E9%98%B5%E8%B5%B7%E6%BA%90%20%E8%B6%85%E5%8D%83%E4%B8%87%E7%BE%8E%E5%85%83%20A%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J6" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -493,21 +493,21 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L6" s="12" t="str">
-        <x:v>为光能源 是一家专注于电力电子 / 固态变压器的企业。</x:v>
+        <x:v>企业级 AI 基础设施公司，围绕数据管理与 AI 计算场景提供技术产品。</x:v>
       </x:c>
       <x:c r="M6" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.matrixorigin.cn/</x:v>
       </x:c>
       <x:c r="N6" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>飞捷科思</x:v>
+        <x:v>为光能源</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>半导体</x:v>
+        <x:v>电力电子 / 固态变压器</x:v>
       </x:c>
       <x:c r="C7" s="13" t="n">
         <x:v>46240.333333333336</x:v>
@@ -516,17 +516,17 @@
         <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>A1 轮</x:v>
+        <x:v>B 轮</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G7" s="14"/>
       <x:c r="H7" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>中国网</x:v>
       </x:c>
       <x:c r="I7" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%A3%9E%E6%8D%B7%E7%A7%91%E6%80%9D%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E4%B8%BA%E5%85%89%E8%83%BD%E6%BA%90%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J7" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -535,7 +535,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L7" s="12" t="str">
-        <x:v>飞捷科思 是一家专注于半导体的企业。</x:v>
+        <x:v>为光能源 是一家专注于电力电子 / 固态变压器的企业。</x:v>
       </x:c>
       <x:c r="M7" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -546,29 +546,29 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>蓝凌星通</x:v>
+        <x:v>飞捷科思</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>卫星通信</x:v>
+        <x:v>半导体</x:v>
       </x:c>
       <x:c r="C8" s="13" t="n">
         <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>股权融资</x:v>
+        <x:v>A1 轮</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G8" s="14"/>
       <x:c r="H8" s="12" t="str">
-        <x:v>启迪之星</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I8" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%93%9D%E5%87%8C%E6%98%9F%E9%80%9A%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%A3%9E%E6%8D%B7%E7%A7%91%E6%80%9D%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J8" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -577,7 +577,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
-        <x:v>蓝凌星通 是一家专注于卫星通信的企业。</x:v>
+        <x:v>飞捷科思 是一家专注于半导体的企业。</x:v>
       </x:c>
       <x:c r="M8" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -588,29 +588,29 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>昉擎科技</x:v>
+        <x:v>蓝凌星通</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>AI 算力芯片</x:v>
+        <x:v>卫星通信</x:v>
       </x:c>
       <x:c r="C9" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>A1 轮</x:v>
+        <x:v>股权融资</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G9" s="14"/>
       <x:c r="H9" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>启迪之星</x:v>
       </x:c>
       <x:c r="I9" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E8%93%9D%E5%87%8C%E6%98%9F%E9%80%9A%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J9" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -619,7 +619,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L9" s="12" t="str">
-        <x:v>昉擎科技 是一家专注于AI 算力芯片的企业。</x:v>
+        <x:v>蓝凌星通 是一家专注于卫星通信的企业。</x:v>
       </x:c>
       <x:c r="M9" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -630,19 +630,19 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>协鑫光电</x:v>
+        <x:v>昉擎科技</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>钙钛矿光伏</x:v>
+        <x:v>AI 算力芯片</x:v>
       </x:c>
       <x:c r="C10" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>超 1 亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>D1 轮</x:v>
+        <x:v>A1 轮</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
         <x:v>CNY</x:v>
@@ -652,7 +652,7 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I10" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J10" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -661,7 +661,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L10" s="12" t="str">
-        <x:v>协鑫光电 是一家专注于钙钛矿光伏的企业。</x:v>
+        <x:v>昉擎科技 是一家专注于AI 算力芯片的企业。</x:v>
       </x:c>
       <x:c r="M10" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -672,31 +672,29 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>主动科技</x:v>
+        <x:v>协鑫光电</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>脑机接口</x:v>
+        <x:v>钙钛矿光伏</x:v>
       </x:c>
       <x:c r="C11" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>3.3 亿元人民币</x:v>
+        <x:v>超 1 亿元人民币</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>D1 轮</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G11" s="14" t="n">
-        <x:v>33000</x:v>
-      </x:c>
+      <x:c r="G11" s="14"/>
       <x:c r="H11" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I11" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J11" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -705,7 +703,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L11" s="12" t="str">
-        <x:v>主动科技 是一家专注于脑机接口的企业。</x:v>
+        <x:v>协鑫光电 是一家专注于钙钛矿光伏的企业。</x:v>
       </x:c>
       <x:c r="M11" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -716,29 +714,31 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>西湖心辰</x:v>
+        <x:v>主动科技</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>生成式 AI</x:v>
+        <x:v>脑机接口</x:v>
       </x:c>
       <x:c r="C12" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>3.3 亿元人民币</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>B+ 轮</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G12" s="14"/>
+      <x:c r="G12" s="14" t="n">
+        <x:v>33000</x:v>
+      </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>澎湃新闻</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J12" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -747,40 +747,40 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
-        <x:v>生成式 AI 公司，聚焦多模态大模型与 AI 原生应用研发。</x:v>
+        <x:v>主动科技 是一家专注于脑机接口的企业。</x:v>
       </x:c>
       <x:c r="M12" s="12" t="str">
-        <x:v>https://www.westlake.ai/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N12" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>璨辰科技</x:v>
+        <x:v>西湖心辰</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>医疗 AI / 虚拟器官仿真</x:v>
+        <x:v>生成式 AI</x:v>
       </x:c>
       <x:c r="C13" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>天使系列轮</x:v>
+        <x:v>B+ 轮</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G13" s="14"/>
       <x:c r="H13" s="12" t="str">
-        <x:v>雷峰网</x:v>
+        <x:v>澎湃新闻</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J13" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -789,42 +789,40 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L13" s="12" t="str">
-        <x:v>璨辰科技 是一家专注于医疗 AI / 虚拟器官仿真的企业。</x:v>
+        <x:v>生成式 AI 公司，聚焦多模态大模型与 AI 原生应用研发。</x:v>
       </x:c>
       <x:c r="M13" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.westlake.ai/</x:v>
       </x:c>
       <x:c r="N13" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>鸿鹄航空</x:v>
+        <x:v>璨辰科技</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>航空航天</x:v>
+        <x:v>医疗 AI / 虚拟器官仿真</x:v>
       </x:c>
       <x:c r="C14" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>7,000 万元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>天使系列轮</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G14" s="14" t="n">
-        <x:v>7000</x:v>
-      </x:c>
+      <x:c r="G14" s="14"/>
       <x:c r="H14" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>雷峰网</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J14" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -833,7 +831,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str">
-        <x:v>鸿鹄航空 是一家专注于航空航天的企业。</x:v>
+        <x:v>璨辰科技 是一家专注于医疗 AI / 虚拟器官仿真的企业。</x:v>
       </x:c>
       <x:c r="M14" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -844,31 +842,31 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>元育生物</x:v>
+        <x:v>鸿鹄航空</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>生物医药</x:v>
+        <x:v>航空航天</x:v>
       </x:c>
       <x:c r="C15" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>亿元人民币</x:v>
+        <x:v>7,000 万元人民币</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G15" s="14" t="n">
-        <x:v>10000</x:v>
+        <x:v>7000</x:v>
       </x:c>
       <x:c r="H15" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I15" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J15" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -877,7 +875,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L15" s="12" t="str">
-        <x:v>元育生物 是一家专注于生物医药的企业。</x:v>
+        <x:v>鸿鹄航空 是一家专注于航空航天的企业。</x:v>
       </x:c>
       <x:c r="M15" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -888,38 +886,40 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>幺正量子</x:v>
+        <x:v>元育生物</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>量子计算</x:v>
+        <x:v>生物医药</x:v>
       </x:c>
       <x:c r="C16" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>亿元人民币</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>A+ 轮</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G16" s="14"/>
+      <x:c r="G16" s="14" t="n">
+        <x:v>10000</x:v>
+      </x:c>
       <x:c r="H16" s="12" t="str">
-        <x:v>大河财立方</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I16" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J16" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K16" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L16" s="12" t="str">
-        <x:v>量子计算技术公司，面向量子软硬件与产业化应用开展研发。</x:v>
+        <x:v>元育生物 是一家专注于生物医药的企业。</x:v>
       </x:c>
       <x:c r="M16" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -930,29 +930,29 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>恺望数据</x:v>
+        <x:v>幺正量子</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>AI 数据服务</x:v>
+        <x:v>量子计算</x:v>
       </x:c>
       <x:c r="C17" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>逾亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G17" s="14"/>
       <x:c r="H17" s="12" t="str">
-        <x:v>封面新闻</x:v>
+        <x:v>大河财立方</x:v>
       </x:c>
       <x:c r="I17" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J17" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -961,7 +961,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L17" s="12" t="str">
-        <x:v>AI 数据服务公司，为具身智能等场景提供数据采集、处理与训练支持。</x:v>
+        <x:v>量子计算技术公司，面向量子软硬件与产业化应用开展研发。</x:v>
       </x:c>
       <x:c r="M17" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -972,29 +972,29 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>求是光谱</x:v>
+        <x:v>恺望数据</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>光谱检测</x:v>
+        <x:v>AI 数据服务</x:v>
       </x:c>
       <x:c r="C18" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
+        <x:v>逾亿元人民币</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="str">
         <x:v>未披露</x:v>
-      </x:c>
-      <x:c r="E18" s="12" t="str">
-        <x:v>B++ 轮</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G18" s="14"/>
       <x:c r="H18" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>封面新闻</x:v>
       </x:c>
       <x:c r="I18" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J18" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -1003,7 +1003,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L18" s="12" t="str">
-        <x:v>光谱检测技术公司，面向工业与科研场景提供光谱相关产品和解决方案。</x:v>
+        <x:v>AI 数据服务公司，为具身智能等场景提供数据采集、处理与训练支持。</x:v>
       </x:c>
       <x:c r="M18" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1014,10 +1014,10 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>熵简科技</x:v>
+        <x:v>求是光谱</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>企业软件 / 数据智能</x:v>
+        <x:v>光谱检测</x:v>
       </x:c>
       <x:c r="C19" s="13" t="n">
         <x:v>46237.333333333336</x:v>
@@ -1026,7 +1026,7 @@
         <x:v>未披露</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>C 轮</x:v>
+        <x:v>B++ 轮</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
         <x:v>CNY</x:v>
@@ -1036,7 +1036,7 @@
         <x:v>新浪财经</x:v>
       </x:c>
       <x:c r="I19" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J19" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -1045,7 +1045,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L19" s="12" t="str">
-        <x:v>企业级技术服务公司，聚焦数据智能与软件产品研发。</x:v>
+        <x:v>光谱检测技术公司，面向工业与科研场景提供光谱相关产品和解决方案。</x:v>
       </x:c>
       <x:c r="M19" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1056,19 +1056,19 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>灏存科技</x:v>
+        <x:v>熵简科技</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>硬科技</x:v>
+        <x:v>企业软件 / 数据智能</x:v>
       </x:c>
       <x:c r="C20" s="13" t="n">
-        <x:v>46235.333333333336</x:v>
+        <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
         <x:v>未披露</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>C 轮</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
         <x:v>CNY</x:v>
@@ -1078,7 +1078,7 @@
         <x:v>新浪财经</x:v>
       </x:c>
       <x:c r="I20" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J20" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -1087,7 +1087,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L20" s="12" t="str">
-        <x:v>硬科技企业，公开报道披露其近期完成 A+ 轮融资。</x:v>
+        <x:v>企业级技术服务公司，聚焦数据智能与软件产品研发。</x:v>
       </x:c>
       <x:c r="M20" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1098,45 +1098,87 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
+        <x:v>灏存科技</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>硬科技</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="n">
+        <x:v>46235.333333333336</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="str">
+        <x:v>A+ 轮</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G21" s="14"/>
+      <x:c r="H21" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I21" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J21" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K21" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L21" s="12" t="str">
+        <x:v>硬科技企业，公开报道披露其近期完成 A+ 轮融资。</x:v>
+      </x:c>
+      <x:c r="M21" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N21" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="12" t="str">
         <x:v>月之暗面（Kimi）</x:v>
       </x:c>
-      <x:c r="B21" s="12" t="str">
+      <x:c r="B22" s="12" t="str">
         <x:v>大模型</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="n">
+      <x:c r="C22" s="13" t="n">
         <x:v>46234.333333333336</x:v>
       </x:c>
-      <x:c r="D21" s="12" t="str">
+      <x:c r="D22" s="12" t="str">
         <x:v>超 35 亿美元</x:v>
       </x:c>
-      <x:c r="E21" s="12" t="str">
+      <x:c r="E22" s="12" t="str">
         <x:v>F 轮</x:v>
       </x:c>
-      <x:c r="F21" s="12" t="str">
+      <x:c r="F22" s="12" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="G21" s="14" t="n">
+      <x:c r="G22" s="14" t="n">
         <x:v>2520000</x:v>
       </x:c>
-      <x:c r="H21" s="12" t="str">
+      <x:c r="H22" s="12" t="str">
         <x:v>创业邦</x:v>
       </x:c>
-      <x:c r="I21" s="16" t="str">
+      <x:c r="I22" s="16" t="str">
         <x:v>https://news.google.com/search?q=%E6%9C%88%E4%B9%8B%E6%9A%97%E9%9D%A2%20F%E8%BD%AE%2035%E4%BA%BF%E7%BE%8E%E5%85%83&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
-      <x:c r="J21" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
-      </x:c>
-      <x:c r="K21" s="12" t="str">
-        <x:v>已核验</x:v>
-      </x:c>
-      <x:c r="L21" s="12" t="str">
+      <x:c r="J22" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K22" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L22" s="12" t="str">
         <x:v>大模型创业公司，推出 Kimi 等面向个人与企业的 AI 产品。</x:v>
       </x:c>
-      <x:c r="M21" s="12" t="str">
+      <x:c r="M22" s="12" t="str">
         <x:v>https://www.moonshot.cn/</x:v>
       </x:c>
-      <x:c r="N21" s="12" t="str">
+      <x:c r="N22" s="12" t="str">
         <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
@@ -1504,10 +1546,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46242.14893152778</x:v>
+        <x:v>46242.1534702662</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C2" t="n">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
data: enrich energy and robotics profiles
</commit_message>
<xml_diff>
--- a/近期融资公司追踪.xlsx
+++ b/近期融资公司追踪.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R7d386a9e909f4105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="R9724e5b4228a4776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R95bc27f6f54e4fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R58bc39e0d8134bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Re552c5ed24c04d7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="Reb3f73bb278a41e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -535,13 +535,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L7" s="12" t="str">
-        <x:v>为光能源 是一家专注于电力电子 / 固态变压器的企业。</x:v>
+        <x:v>西安为光能源科技有限公司，面向算力中心、电动交通、新型配网和储能等场景，围绕固态变压器（SST）等新型电力电子装备提供能源互联网解决方案。</x:v>
       </x:c>
       <x:c r="M7" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.weiguangenergy.com/portal/about/index.html</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>服务热线：400-868-6988；地址：陕西省西安市高新区毕原二路3号先导院南区5-6号楼；公众号：WGenergy；在线留言：官网联系页面。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -630,61 +630,61 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>昉擎科技</x:v>
+        <x:v>RoboParty（萝博派对）</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>AI 算力芯片</x:v>
+        <x:v>具身智能 / 人形机器人</x:v>
       </x:c>
       <x:c r="C10" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46238.333333333336</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>近 5 亿元人民币</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>A1 轮</x:v>
+        <x:v>天使++轮及 Pre-A 轮</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G10" s="14"/>
       <x:c r="H10" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>快科技（新浪财经转载）</x:v>
       </x:c>
       <x:c r="I10" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-04/doc-inimchzp5821502.shtml</x:v>
       </x:c>
       <x:c r="J10" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46242.5</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L10" s="12" t="str">
-        <x:v>昉擎科技 是一家专注于AI 算力芯片的企业。</x:v>
+        <x:v>上海萝博派对科技有限公司，专注全栈开源双足人形机器人；其公开项目覆盖机器人结构、电气、训练和部署。</x:v>
       </x:c>
       <x:c r="M10" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://github.com/Roboparty</x:v>
       </x:c>
       <x:c r="N10" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>未见公开商务电话或邮箱；开源技术交流 QQ 群：546376843；官方 GitHub：github.com/Roboparty。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>协鑫光电</x:v>
+        <x:v>昉擎科技</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>钙钛矿光伏</x:v>
+        <x:v>AI 算力芯片</x:v>
       </x:c>
       <x:c r="C11" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>超 1 亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>D1 轮</x:v>
+        <x:v>A1 轮</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
         <x:v>CNY</x:v>
@@ -694,7 +694,7 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I11" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J11" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -703,7 +703,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L11" s="12" t="str">
-        <x:v>协鑫光电 是一家专注于钙钛矿光伏的企业。</x:v>
+        <x:v>昉擎科技 是一家专注于AI 算力芯片的企业。</x:v>
       </x:c>
       <x:c r="M11" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -714,31 +714,29 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>主动科技</x:v>
+        <x:v>协鑫光电</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>脑机接口</x:v>
+        <x:v>钙钛矿光伏</x:v>
       </x:c>
       <x:c r="C12" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>3.3 亿元人民币</x:v>
+        <x:v>超 1 亿元人民币</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>D1 轮</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G12" s="14" t="n">
-        <x:v>33000</x:v>
-      </x:c>
+      <x:c r="G12" s="14"/>
       <x:c r="H12" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J12" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -747,7 +745,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
-        <x:v>主动科技 是一家专注于脑机接口的企业。</x:v>
+        <x:v>协鑫光电 是一家专注于钙钛矿光伏的企业。</x:v>
       </x:c>
       <x:c r="M12" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -758,29 +756,31 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>西湖心辰</x:v>
+        <x:v>主动科技</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>生成式 AI</x:v>
+        <x:v>脑机接口</x:v>
       </x:c>
       <x:c r="C13" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>3.3 亿元人民币</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>B+ 轮</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G13" s="14"/>
+      <x:c r="G13" s="14" t="n">
+        <x:v>33000</x:v>
+      </x:c>
       <x:c r="H13" s="12" t="str">
-        <x:v>澎湃新闻</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J13" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -789,40 +789,40 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L13" s="12" t="str">
-        <x:v>生成式 AI 公司，聚焦多模态大模型与 AI 原生应用研发。</x:v>
+        <x:v>主动科技 是一家专注于脑机接口的企业。</x:v>
       </x:c>
       <x:c r="M13" s="12" t="str">
-        <x:v>https://www.westlake.ai/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N13" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>璨辰科技</x:v>
+        <x:v>西湖心辰</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>医疗 AI / 虚拟器官仿真</x:v>
+        <x:v>生成式 AI</x:v>
       </x:c>
       <x:c r="C14" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>天使系列轮</x:v>
+        <x:v>B+ 轮</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G14" s="14"/>
       <x:c r="H14" s="12" t="str">
-        <x:v>雷峰网</x:v>
+        <x:v>澎湃新闻</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J14" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -831,42 +831,40 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str">
-        <x:v>璨辰科技 是一家专注于医疗 AI / 虚拟器官仿真的企业。</x:v>
+        <x:v>生成式 AI 公司，聚焦多模态大模型与 AI 原生应用研发。</x:v>
       </x:c>
       <x:c r="M14" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.westlake.ai/</x:v>
       </x:c>
       <x:c r="N14" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>鸿鹄航空</x:v>
+        <x:v>璨辰科技</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>航空航天</x:v>
+        <x:v>医疗 AI / 虚拟器官仿真</x:v>
       </x:c>
       <x:c r="C15" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>7,000 万元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>天使系列轮</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G15" s="14" t="n">
-        <x:v>7000</x:v>
-      </x:c>
+      <x:c r="G15" s="14"/>
       <x:c r="H15" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>雷峰网</x:v>
       </x:c>
       <x:c r="I15" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J15" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -875,7 +873,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L15" s="12" t="str">
-        <x:v>鸿鹄航空 是一家专注于航空航天的企业。</x:v>
+        <x:v>璨辰科技 是一家专注于医疗 AI / 虚拟器官仿真的企业。</x:v>
       </x:c>
       <x:c r="M15" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -886,31 +884,31 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>元育生物</x:v>
+        <x:v>鸿鹄航空</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>生物医药</x:v>
+        <x:v>航空航天</x:v>
       </x:c>
       <x:c r="C16" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>亿元人民币</x:v>
+        <x:v>7,000 万元人民币</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G16" s="14" t="n">
-        <x:v>10000</x:v>
+        <x:v>7000</x:v>
       </x:c>
       <x:c r="H16" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I16" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J16" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -919,7 +917,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L16" s="12" t="str">
-        <x:v>元育生物 是一家专注于生物医药的企业。</x:v>
+        <x:v>鸿鹄航空 是一家专注于航空航天的企业。</x:v>
       </x:c>
       <x:c r="M16" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -930,38 +928,40 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>幺正量子</x:v>
+        <x:v>元育生物</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>量子计算</x:v>
+        <x:v>生物医药</x:v>
       </x:c>
       <x:c r="C17" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>亿元人民币</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>A+ 轮</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G17" s="14"/>
+      <x:c r="G17" s="14" t="n">
+        <x:v>10000</x:v>
+      </x:c>
       <x:c r="H17" s="12" t="str">
-        <x:v>大河财立方</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I17" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J17" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K17" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L17" s="12" t="str">
-        <x:v>量子计算技术公司，面向量子软硬件与产业化应用开展研发。</x:v>
+        <x:v>元育生物 是一家专注于生物医药的企业。</x:v>
       </x:c>
       <x:c r="M17" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -972,29 +972,29 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>恺望数据</x:v>
+        <x:v>幺正量子</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>AI 数据服务</x:v>
+        <x:v>量子计算</x:v>
       </x:c>
       <x:c r="C18" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>逾亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G18" s="14"/>
       <x:c r="H18" s="12" t="str">
-        <x:v>封面新闻</x:v>
+        <x:v>大河财立方</x:v>
       </x:c>
       <x:c r="I18" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J18" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -1003,7 +1003,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L18" s="12" t="str">
-        <x:v>AI 数据服务公司，为具身智能等场景提供数据采集、处理与训练支持。</x:v>
+        <x:v>量子计算技术公司，面向量子软硬件与产业化应用开展研发。</x:v>
       </x:c>
       <x:c r="M18" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1014,29 +1014,29 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>求是光谱</x:v>
+        <x:v>恺望数据</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>光谱检测</x:v>
+        <x:v>AI 数据服务</x:v>
       </x:c>
       <x:c r="C19" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
+        <x:v>逾亿元人民币</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="str">
         <x:v>未披露</x:v>
-      </x:c>
-      <x:c r="E19" s="12" t="str">
-        <x:v>B++ 轮</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G19" s="14"/>
       <x:c r="H19" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>封面新闻</x:v>
       </x:c>
       <x:c r="I19" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J19" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -1045,7 +1045,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L19" s="12" t="str">
-        <x:v>光谱检测技术公司，面向工业与科研场景提供光谱相关产品和解决方案。</x:v>
+        <x:v>AI 数据服务公司，为具身智能等场景提供数据采集、处理与训练支持。</x:v>
       </x:c>
       <x:c r="M19" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1056,10 +1056,10 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>熵简科技</x:v>
+        <x:v>求是光谱</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>企业软件 / 数据智能</x:v>
+        <x:v>光谱检测</x:v>
       </x:c>
       <x:c r="C20" s="13" t="n">
         <x:v>46237.333333333336</x:v>
@@ -1068,7 +1068,7 @@
         <x:v>未披露</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>C 轮</x:v>
+        <x:v>B++ 轮</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
         <x:v>CNY</x:v>
@@ -1078,7 +1078,7 @@
         <x:v>新浪财经</x:v>
       </x:c>
       <x:c r="I20" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J20" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -1087,7 +1087,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L20" s="12" t="str">
-        <x:v>企业级技术服务公司，聚焦数据智能与软件产品研发。</x:v>
+        <x:v>光谱检测技术公司，面向工业与科研场景提供光谱相关产品和解决方案。</x:v>
       </x:c>
       <x:c r="M20" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1098,19 +1098,19 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>灏存科技</x:v>
+        <x:v>熵简科技</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>硬科技</x:v>
+        <x:v>企业软件 / 数据智能</x:v>
       </x:c>
       <x:c r="C21" s="13" t="n">
-        <x:v>46235.333333333336</x:v>
+        <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
         <x:v>未披露</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>C 轮</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
         <x:v>CNY</x:v>
@@ -1120,7 +1120,7 @@
         <x:v>新浪财经</x:v>
       </x:c>
       <x:c r="I21" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J21" s="15" t="n">
         <x:v>46242.479166666664</x:v>
@@ -1129,7 +1129,7 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L21" s="12" t="str">
-        <x:v>硬科技企业，公开报道披露其近期完成 A+ 轮融资。</x:v>
+        <x:v>企业级技术服务公司，聚焦数据智能与软件产品研发。</x:v>
       </x:c>
       <x:c r="M21" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1140,45 +1140,87 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
+        <x:v>灏存科技</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="str">
+        <x:v>硬科技</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="n">
+        <x:v>46235.333333333336</x:v>
+      </x:c>
+      <x:c r="D22" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E22" s="12" t="str">
+        <x:v>A+ 轮</x:v>
+      </x:c>
+      <x:c r="F22" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G22" s="14"/>
+      <x:c r="H22" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I22" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J22" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K22" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L22" s="12" t="str">
+        <x:v>硬科技企业，公开报道披露其近期完成 A+ 轮融资。</x:v>
+      </x:c>
+      <x:c r="M22" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N22" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="12" t="str">
         <x:v>月之暗面（Kimi）</x:v>
       </x:c>
-      <x:c r="B22" s="12" t="str">
+      <x:c r="B23" s="12" t="str">
         <x:v>大模型</x:v>
       </x:c>
-      <x:c r="C22" s="13" t="n">
+      <x:c r="C23" s="13" t="n">
         <x:v>46234.333333333336</x:v>
       </x:c>
-      <x:c r="D22" s="12" t="str">
+      <x:c r="D23" s="12" t="str">
         <x:v>超 35 亿美元</x:v>
       </x:c>
-      <x:c r="E22" s="12" t="str">
+      <x:c r="E23" s="12" t="str">
         <x:v>F 轮</x:v>
       </x:c>
-      <x:c r="F22" s="12" t="str">
+      <x:c r="F23" s="12" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="G22" s="14" t="n">
+      <x:c r="G23" s="14" t="n">
         <x:v>2520000</x:v>
       </x:c>
-      <x:c r="H22" s="12" t="str">
+      <x:c r="H23" s="12" t="str">
         <x:v>创业邦</x:v>
       </x:c>
-      <x:c r="I22" s="16" t="str">
+      <x:c r="I23" s="16" t="str">
         <x:v>https://news.google.com/search?q=%E6%9C%88%E4%B9%8B%E6%9A%97%E9%9D%A2%20F%E8%BD%AE%2035%E4%BA%BF%E7%BE%8E%E5%85%83&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
-      <x:c r="J22" s="15" t="n">
+      <x:c r="J23" s="15" t="n">
         <x:v>46241.479166666664</x:v>
       </x:c>
-      <x:c r="K22" s="12" t="str">
-        <x:v>已核验</x:v>
-      </x:c>
-      <x:c r="L22" s="12" t="str">
+      <x:c r="K23" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L23" s="12" t="str">
         <x:v>大模型创业公司，推出 Kimi 等面向个人与企业的 AI 产品。</x:v>
       </x:c>
-      <x:c r="M22" s="12" t="str">
+      <x:c r="M23" s="12" t="str">
         <x:v>https://www.moonshot.cn/</x:v>
       </x:c>
-      <x:c r="N22" s="12" t="str">
+      <x:c r="N23" s="12" t="str">
         <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
@@ -1546,10 +1588,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46242.1534702662</x:v>
+        <x:v>46242.15577440972</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C2" t="n">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
feat: expand company profiles
</commit_message>
<xml_diff>
--- a/近期融资公司追踪.xlsx
+++ b/近期融资公司追踪.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R58bc39e0d8134bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Re552c5ed24c04d7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="Reb3f73bb278a41e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R3e96ab7aac684d2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="R154d6f1729c14dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R823804b89c914e09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -449,7 +449,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L5" s="12" t="str">
-        <x:v>AI 视频大模型产品，面向内容创作和商业化视频生成场景提供服务。</x:v>
+        <x:v>可灵 AI 是面向视频生成与创作的 AI 大模型产品，支持文本、图片等输入驱动的视频内容生成和编辑。产品服务广告创意、影视内容、社交媒体和商业化营销等场景，重点提升视频生成的一致性、可控性和创作效率。</x:v>
       </x:c>
       <x:c r="M5" s="12" t="str">
         <x:v>https://klingai.com/</x:v>
@@ -493,13 +493,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L6" s="12" t="str">
-        <x:v>企业级 AI 基础设施公司，围绕数据管理与 AI 计算场景提供技术产品。</x:v>
+        <x:v>矩阵起源专注 AI 原生数据基础设施，提供多模态数据处理、数据库与企业级 AI 数据底座产品及解决方案。其产品面向企业在结构化、非结构化和向量数据之间建立统一的数据管理与计算能力，为模型训练、知识检索和 AI 应用部署提供底层支撑。</x:v>
       </x:c>
       <x:c r="M6" s="12" t="str">
-        <x:v>https://www.matrixorigin.cn/</x:v>
+        <x:v>https://matrixorigin.cn/</x:v>
       </x:c>
       <x:c r="N6" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>商务邮箱：contact@matrixorigin.cn。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -535,13 +535,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L7" s="12" t="str">
-        <x:v>西安为光能源科技有限公司，面向算力中心、电动交通、新型配网和储能等场景，围绕固态变压器（SST）等新型电力电子装备提供能源互联网解决方案。</x:v>
+        <x:v>西安为光能源科技有限公司聚焦固态变压器（SST）等新型电力电子装备及能源互联网解决方案。公司瞄准算力中心、电动交通、新型配网和储能等高功率密度场景，通过电能变换、控制和系统集成提升供配电效率与灵活性。</x:v>
       </x:c>
       <x:c r="M7" s="12" t="str">
-        <x:v>https://www.weiguangenergy.com/portal/about/index.html</x:v>
+        <x:v>https://www.weiguangenergy.com/</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
-        <x:v>服务热线：400-868-6988；地址：陕西省西安市高新区毕原二路3号先导院南区5-6号楼；公众号：WGenergy；在线留言：官网联系页面。</x:v>
+        <x:v>服务热线：400-868-6988；商务邮箱（官网公开）：wangjuan0509@foxmail.com；地址：陕西省西安市高新区毕原二路3号先导院南区5-6号楼；公众号：WGenergy；在线留言：官网联系页。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -577,13 +577,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
-        <x:v>飞捷科思 是一家专注于半导体的企业。</x:v>
+        <x:v>飞捷科思以高精度实时物理仿真引擎为核心，研发面向具身智能和人形机器人的物理智能技术与产品。其能力重点在于让机器人在虚拟环境中完成动力学、接触和运动策略验证，以缩短从算法训练到真实机器部署的迭代周期。</x:v>
       </x:c>
       <x:c r="M8" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://fysics.net/</x:v>
       </x:c>
       <x:c r="N8" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>电话：021-60197571；商务邮箱：fysics@fysics.ai；官网联系页：https://fysics.net/contact.html。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -619,13 +619,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L9" s="12" t="str">
-        <x:v>蓝凌星通 是一家专注于卫星通信的企业。</x:v>
+        <x:v>蓝凌星通是蓝牙卫星系统服务商，利用低轨卫星为蓝牙终端提供低成本、低功耗的物联网连接和行业监测方案。其目标是把现有蓝牙终端延伸到传统地面网络覆盖不足的区域，服务户外、物流、资产追踪和行业监测等场景。</x:v>
       </x:c>
       <x:c r="M9" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.bluelinksatcom.com/</x:v>
       </x:c>
       <x:c r="N9" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>电话：400-8818-251；商务邮箱：market@bluelinksatcom.com。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -661,13 +661,13 @@
         <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L10" s="12" t="str">
-        <x:v>上海萝博派对科技有限公司，专注全栈开源双足人形机器人；其公开项目覆盖机器人结构、电气、训练和部署。</x:v>
+        <x:v>RoboParty 专注低成本、高性能双足人形机器人研发，并通过全栈开源建设机器人开发生态。公司公开机器人结构、电气、训练和部署等技术资料，希望降低研究者与开发者进入人形机器人研发的门槛，并推动软硬件协同迭代。</x:v>
       </x:c>
       <x:c r="M10" s="12" t="str">
-        <x:v>https://github.com/Roboparty</x:v>
+        <x:v>https://roboparty.com/</x:v>
       </x:c>
       <x:c r="N10" s="12" t="str">
-        <x:v>未见公开商务电话或邮箱；开源技术交流 QQ 群：546376843；官方 GitHub：github.com/Roboparty。</x:v>
+        <x:v>商务邮箱：contact@roboparty.com；开源技术交流 QQ 群：1078670917；官方 GitHub：https://github.com/Roboparty。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -703,7 +703,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L11" s="12" t="str">
-        <x:v>昉擎科技 是一家专注于AI 算力芯片的企业。</x:v>
+        <x:v>昉擎科技是新一代智能计算系统企业，基于分离式架构和 4D Memory 理论，自主研发芯片、硬件系统与软件栈。公司重点解决 AI 计算系统的通用性、扩展性与工程化部署问题；本轮融资主要用于自研芯片和系统研发、规模化量产、软件生态建设及人才引进。</x:v>
       </x:c>
       <x:c r="M11" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -745,13 +745,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
-        <x:v>协鑫光电 是一家专注于钙钛矿光伏的企业。</x:v>
+        <x:v>协鑫光电主要从事大面积钙钛矿光伏组件的研发、生产及商业化应用。公司围绕钙钛矿材料、组件制备、封装可靠性和量产工艺推进技术迭代，面向下一代高效率光伏组件及其应用市场。</x:v>
       </x:c>
       <x:c r="M12" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.gcl-perovskite.com/</x:v>
       </x:c>
       <x:c r="N12" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网公开电话：86-0512-57562287；官网联系页：https://www.gcl-power.com/contact.html。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -789,7 +789,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L13" s="12" t="str">
-        <x:v>主动科技 是一家专注于脑机接口的企业。</x:v>
+        <x:v>主动科技是一家侵入式脑机接口技术研发与产业化企业，核心产品为“天枢”运动脑机接口。公开报道显示，公司成立于 2026 年 2 月，正推进高通道脑机系统、微纳加工平台与临床试验，目标是推动侵入式脑机接口从实验室验证走向医疗器械产业化。</x:v>
       </x:c>
       <x:c r="M13" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -831,13 +831,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str">
-        <x:v>生成式 AI 公司，聚焦多模态大模型与 AI 原生应用研发。</x:v>
+        <x:v>西湖心辰是一家生成式 AI 公司，研发西湖大模型及面向创作与企业场景的 AI 原生应用。公司将大模型能力用于内容生成、智能交互和行业工作流，强调模型能力与实际产品体验、企业落地场景的结合。</x:v>
       </x:c>
       <x:c r="M14" s="12" t="str">
-        <x:v>https://www.westlake.ai/</x:v>
+        <x:v>https://xinchenai.com/</x:v>
       </x:c>
       <x:c r="N14" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>电话：400-8126-618；邮箱：support@xinchenai.com；地址：浙江省杭州市西湖区智强路428号云创镓谷6号楼6楼604室。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -873,7 +873,7 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L15" s="12" t="str">
-        <x:v>璨辰科技 是一家专注于医疗 AI / 虚拟器官仿真的企业。</x:v>
+        <x:v>璨辰科技聚焦系统级虚拟器官时空动态演化模型研发，构建从分子、细胞、组织到器官的全尺度 AI 数字孪生平台。其方案服务于新药临床前评价、发育毒性评估与疾病机制研究，并通过“仿真—湿实验—临床前验证”的数据闭环提升模型的产业转化价值。</x:v>
       </x:c>
       <x:c r="M15" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -917,13 +917,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L16" s="12" t="str">
-        <x:v>鸿鹄航空 是一家专注于航空航天的企业。</x:v>
+        <x:v>青岛鸿鹄航空科技有限公司专注航空温控产品与服务，是海尔生物医疗控股子公司。公司围绕航空装备温度控制和相关系统服务开展产品研发，服务航空运行与专业运输等对环境控制要求较高的场景。</x:v>
       </x:c>
       <x:c r="M16" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.hbtempconaviation.com/</x:v>
       </x:c>
       <x:c r="N16" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>电话：+86-400-863-0863；邮箱：aviation@haierbiomedical.com；地址：青岛市高新区丰源路280号。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -961,13 +961,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L17" s="12" t="str">
-        <x:v>元育生物 是一家专注于生物医药的企业。</x:v>
+        <x:v>元育生物是微藻生物合成企业，开发可持续微藻基原料并提供定制化应用解决方案。公司以微藻培养、代谢调控和生物制造为技术基础，探索在食品营养、功能原料、日化与绿色消费品等领域的产业化应用。</x:v>
       </x:c>
       <x:c r="M17" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.protoga.com/</x:v>
       </x:c>
       <x:c r="N17" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>珠海：0756-8699334；北京：010-67866793；海外 BD：bd@protoga.com；国内销售：sales@protoga.com；地址：广东省珠海市香洲区南屏镇科技工业园屏北一路30号1栋2楼。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -1003,13 +1003,13 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L18" s="12" t="str">
-        <x:v>量子计算技术公司，面向量子软硬件与产业化应用开展研发。</x:v>
+        <x:v>幺正量子是一家离子阱量子计算企业，提供量子计算系统、设备器件、云服务和行业解决方案。公司围绕离子阱硬件、量子控制、算法与行业应用推进全栈研发，服务科研、教育和量子计算产业化需求。</x:v>
       </x:c>
       <x:c r="M18" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.unitqc.com/</x:v>
       </x:c>
       <x:c r="N18" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>商务邮箱：business@unitqc.com；电话：15391985489；地址：安徽省合肥市高新区望江西路900号中安创谷科技园一期B1栋1-2层。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -1045,13 +1045,13 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L19" s="12" t="str">
-        <x:v>AI 数据服务公司，为具身智能等场景提供数据采集、处理与训练支持。</x:v>
+        <x:v>恺望数据为车企、自动驾驶及 AI 企业提供一站式数据解决方案和自动化数据生产能力。其服务覆盖数据采集、清洗、标注、质检和管理，重点支持自动驾驶、具身智能与大模型训练中的规模化高质量数据供给。</x:v>
       </x:c>
       <x:c r="M19" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://admin.d.konvery.com/</x:v>
       </x:c>
       <x:c r="N19" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官方产品平台：https://admin.d.konvery.com/；官网未公开完整商务电话或邮箱，可通过平台申请试用或联系。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -1087,13 +1087,13 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L20" s="12" t="str">
-        <x:v>光谱检测技术公司，面向工业与科研场景提供光谱相关产品和解决方案。</x:v>
+        <x:v>求是光谱从事多光谱成像芯片、光谱应用方案及光谱大数据研发，为智能终端、汽车电子、医疗和环境监测等场景提供产品与服务。公司将光谱感知能力嵌入硬件和软件方案，用于物质识别、成分分析和复杂环境下的智能检测。</x:v>
       </x:c>
       <x:c r="M20" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.qsspec.com/</x:v>
       </x:c>
       <x:c r="N20" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>电话：0431-88882290；商务联系人：冯硕，18343025432，fengshuo@qsspec.com；展会公开邮箱：hanying@qsspec.com。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -1129,13 +1129,13 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L21" s="12" t="str">
-        <x:v>企业级技术服务公司，聚焦数据智能与软件产品研发。</x:v>
+        <x:v>熵简科技是面向金融资管行业的数字基础设施与数据智能服务商，提供另类数据、知识图谱和全域数据中台等能力。公司自主研发大数据分析引擎，帮助金融机构处理多源异构数据、构建标准化 API，并支持投研、风险管理和业务决策工作流。</x:v>
       </x:c>
       <x:c r="M21" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.valuesimplex.com/</x:v>
       </x:c>
       <x:c r="N21" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网提供业务咨询入口；暂未检索到可交叉确认的公开商务电话或邮箱。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -1171,13 +1171,13 @@
         <x:v>待官网交叉核验</x:v>
       </x:c>
       <x:c r="L22" s="12" t="str">
-        <x:v>硬科技企业，公开报道披露其近期完成 A+ 轮融资。</x:v>
+        <x:v>灏存科技从事人工智能穿戴型肢体动作识别软硬件技术研发，应用于 VR/AR/MR、电影工业和人形机器人运动感知场景。公司以穿戴式传感、人体动作捕捉和算法识别为核心，使虚拟交互、数字内容生产和机器人训练获得更细粒度的运动数据。</x:v>
       </x:c>
       <x:c r="M22" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.hexacercle.com/</x:v>
       </x:c>
       <x:c r="N22" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>商务合作：+86 13349933396；邮箱：mike@hexacercle.com；武汉总部：武汉东湖高新区关东街道华工园三路湖北青创园4栋801。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -1215,13 +1215,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L23" s="12" t="str">
-        <x:v>大模型创业公司，推出 Kimi 等面向个人与企业的 AI 产品。</x:v>
+        <x:v>月之暗面是一家大模型创业公司，推出 Kimi 等面向个人与企业的 AI 产品。其产品以长上下文理解、资料阅读、信息整理和多轮对话为主要能力，覆盖个人效率工具与企业级 AI 应用需求。</x:v>
       </x:c>
       <x:c r="M23" s="12" t="str">
         <x:v>https://www.moonshot.cn/</x:v>
       </x:c>
       <x:c r="N23" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>产品/售后：support@moonshot.cn；媒体：pr@kimi.com；投资者联系：ir@kimi.com；企业微信客服：微信公众号「月之暗面Kimi」菜单“联系我们”。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1368,13 +1368,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L5" s="12" t="str">
-        <x:v>Lumilens 是一家专注于光网络的企业。</x:v>
+        <x:v>Lumilens 为 AI 基础设施提供规模扩展和规模内互连的下一代光子互连产品。公司面向高性能计算和大规模训练集群，尝试以更高带宽、更低功耗的光互连缓解 GPU、交换网络和数据中心内部通信的瓶颈。</x:v>
       </x:c>
       <x:c r="M5" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://lumilens.com/</x:v>
       </x:c>
       <x:c r="N5" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网未公开列出商务邮箱或电话；可通过官网产品/新闻页面关注后续联系入口。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1412,13 +1412,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L6" s="12" t="str">
-        <x:v>Valar Atomics 是一家专注于核能的企业。</x:v>
+        <x:v>Valar Atomics 面向重工业供能、数据中心电力、氢能和清洁燃料场景研发高温气冷堆核能系统。公司重点探索能够规模化制造的先进核能设备，以为高温工业过程和持续增长的算力负荷提供稳定的零碳能源。</x:v>
       </x:c>
       <x:c r="M6" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://valaratomics.com/</x:v>
       </x:c>
       <x:c r="N6" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网提供“Contact us”联系入口；未检索到公开商务邮箱或电话。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1456,13 +1456,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L7" s="12" t="str">
-        <x:v>OLIX 是一家专注于AI 芯片的企业。</x:v>
+        <x:v>OLIX 为前沿 AI 推理构建从芯片、激光器到互连网络的一体化基础设施。公司聚焦计算、光电器件和高速互连的协同设计，目标是提升大模型推理集群的吞吐、能效与扩展能力。</x:v>
       </x:c>
       <x:c r="M7" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://olix.com/</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>媒体/商务邮箱：press@olix.com；公关联系人：olix@strandpartners.com。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1500,13 +1500,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
-        <x:v>网络安全公司，提供以攻击路径验证为核心的安全测试与风险评估产品。</x:v>
+        <x:v>Horizon3.ai 是一家网络安全公司，提供以攻击路径验证为核心的安全测试与风险评估产品。其 NodeZero 平台通过自动化模拟攻击帮助安全团队识别可被实际利用的薄弱点，并将风险发现与修复优先级连接起来。</x:v>
       </x:c>
       <x:c r="M8" s="12" t="str">
         <x:v>https://www.horizon3.ai/</x:v>
       </x:c>
       <x:c r="N8" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>通用咨询：info@horizon3.ai；电话：+1 650-445-4457；媒体：press@horizon3.ai；官网联系页：https://horizon3.ai/contact-us/。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1544,13 +1544,13 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L9" s="12" t="str">
-        <x:v>AI Agent 安全公司，帮助企业识别和管控生成式 AI 与智能体的安全风险。</x:v>
+        <x:v>Zenity 专注 AI Agent 安全，帮助企业识别和管控生成式 AI、低代码工具及智能体带来的数据与权限风险。其产品面向企业安全团队提供资产发现、策略治理和持续监控能力，支持在不阻断业务创新的前提下部署 AI 应用。</x:v>
       </x:c>
       <x:c r="M9" s="12" t="str">
         <x:v>https://www.zenity.io/</x:v>
       </x:c>
       <x:c r="N9" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>商务邮箱：hello@zenity.io；官网联系页：https://zenity.io/company/contact。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1588,7 +1588,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46242.15577440972</x:v>
+        <x:v>46242.248176284724</x:v>
       </x:c>
       <x:c r="B2" t="n">
         <x:v>19</x:v>

</xml_diff>

<commit_message>
fix: support direct local site opening
</commit_message>
<xml_diff>
--- a/近期融资公司追踪.xlsx
+++ b/近期融资公司追踪.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R3e96ab7aac684d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="R154d6f1729c14dea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R823804b89c914e09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="Rfcc1fc3b5a09454e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rd4fc22d632c54eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R7cdda3aaa1614284"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1588,7 +1588,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46242.248176284724</x:v>
+        <x:v>46242.25224228009</x:v>
       </x:c>
       <x:c r="B2" t="n">
         <x:v>19</x:v>

</xml_diff>